<commit_message>
Update game design workbook to latest revision
</commit_message>
<xml_diff>
--- a/data/excel/Thiết kế game.xlsx
+++ b/data/excel/Thiết kế game.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Giai đoạn phát triên" sheetId="2" r:id="rId2"/>
     <sheet name="Combat mechanic" sheetId="3" r:id="rId3"/>
     <sheet name="Term" sheetId="4" r:id="rId4"/>
-    <sheet name="Combat power" sheetId="10" r:id="rId5"/>
+    <sheet name="dummy Combat power" sheetId="10" r:id="rId5"/>
     <sheet name="Item" sheetId="9" r:id="rId6"/>
     <sheet name="Formula" sheetId="5" r:id="rId7"/>
     <sheet name="status" sheetId="7" r:id="rId8"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="756" uniqueCount="575">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="582">
   <si>
     <t>Tên game</t>
   </si>
@@ -1829,7 +1829,7 @@
     <t>Full line</t>
   </si>
   <si>
-    <t>Subtarget 1: -50%. Sub target 2: -25%</t>
+    <t>Subtarget 1: -50%. Sub target 2: -75%</t>
   </si>
   <si>
     <t>Base Penetration chance</t>
@@ -1878,6 +1878,71 @@
   </si>
   <si>
     <t>Base Critical damage bonus</t>
+  </si>
+  <si>
+    <t>Each character has four equipment slots: one weapon slot, equipped with one of the available weapon types; one body armor slot; one accessory slot; and one off-hand slot, equipped with exactly one of the following: Rune Enhancement, Shield, Focus, or Ammunition. Only one item can occupy each slot.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Attack Target determines which enemies may be selected as the primary target: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Front</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> allows only the frontmost living enemy in each column, while </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Any</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> allows any living enemy, including protected enemies and the main character. </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Area of Attack determines which additional positions are hit: Single affects only the primary target; Row Adjacent also hits immediately adjacent positions in the same row; Line Adjacent also hits the position immediately behind the primary target in the same column; Full Line hits the primary target and all positions behind it in that column; and Cross also hits immediately adjacent positions above, below, left, and right. </t>
+  </si>
+  <si>
+    <t>The primary target uses 100% Attack; each secondary target uses the listed Attack modifier before its own mitigation is calculated—for example, −50% means 50% Attack and −25% means 75% Attack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Empty positions and defeated targets are skipped without redistributing damage. </t>
+  </si>
+  <si>
+    <t>The attack area remains fixed around the primary target’s original position for all hits: if the primary target dies, subsequent hits still affect surviving secondary targets without selecting a new primary target.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> If either main character dies, the battle ends immediately and all remaining hits are canceled.</t>
   </si>
   <si>
     <t>Status</t>
@@ -6056,7 +6121,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7142857142857" style="5" customWidth="1"/>
@@ -6239,18 +6304,18 @@
       </c>
       <c r="F7" s="15">
         <f>I7/H7</f>
-        <v>1964.28571428571</v>
+        <v>2678.57142857143</v>
       </c>
       <c r="G7" s="16">
         <f>F7/1000</f>
-        <v>1.96428571428571</v>
+        <v>2.67857142857143</v>
       </c>
       <c r="H7" s="17">
         <v>8.4</v>
       </c>
       <c r="I7" s="15">
-        <f>17900-I8</f>
-        <v>16500</v>
+        <f>17900-I8-I9</f>
+        <v>22500</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -6716,10 +6781,7 @@
       <c r="F27" s="29">
         <v>0.2</v>
       </c>
-      <c r="G27" s="16">
-        <f>F27/1000</f>
-        <v>0.0002</v>
-      </c>
+      <c r="G27" s="16"/>
       <c r="H27" s="17">
         <v>140</v>
       </c>
@@ -6804,7 +6866,7 @@
       <c r="C31" s="13"/>
       <c r="D31" s="14"/>
       <c r="E31" s="15" t="s">
-        <v>515</v>
+        <v>510</v>
       </c>
       <c r="F31" s="28">
         <f>I31/H31</f>
@@ -6981,6 +7043,41 @@
       </c>
       <c r="I39" s="15">
         <v>6000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1">
+      <c r="A43" s="4" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44" s="5" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1">
+      <c r="A45" s="5" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1">
+      <c r="A46" s="5" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1">
+      <c r="A47" s="5" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1">
+      <c r="A48" s="5" t="s">
+        <v>526</v>
       </c>
     </row>
   </sheetData>
@@ -7066,130 +7163,130 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>520</v>
+        <v>527</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>521</v>
+        <v>528</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>522</v>
+        <v>529</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
-        <v>523</v>
+        <v>530</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2" t="s">
-        <v>524</v>
+        <v>531</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>525</v>
+        <v>532</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>526</v>
+        <v>533</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="2" t="s">
-        <v>527</v>
+        <v>534</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>528</v>
+        <v>535</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="2" t="s">
-        <v>529</v>
+        <v>536</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>530</v>
+        <v>537</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="2" t="s">
-        <v>531</v>
+        <v>538</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>532</v>
+        <v>539</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="2" t="s">
-        <v>533</v>
+        <v>540</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2" t="s">
-        <v>534</v>
+        <v>541</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="2" t="s">
-        <v>535</v>
+        <v>542</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
-        <v>536</v>
+        <v>543</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="2" t="s">
-        <v>537</v>
+        <v>544</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2" t="s">
-        <v>538</v>
+        <v>545</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="2" t="s">
-        <v>539</v>
+        <v>546</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2" t="s">
-        <v>540</v>
+        <v>547</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="2" t="s">
-        <v>541</v>
+        <v>548</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2" t="s">
-        <v>542</v>
+        <v>549</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="2" t="s">
-        <v>543</v>
+        <v>550</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2" t="s">
-        <v>544</v>
+        <v>551</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="2" t="s">
-        <v>545</v>
+        <v>552</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2" t="s">
-        <v>546</v>
+        <v>553</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="2" t="s">
-        <v>547</v>
+        <v>554</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2" t="s">
-        <v>548</v>
+        <v>555</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -7200,16 +7297,16 @@
         <v>5</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>549</v>
+        <v>556</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="2" t="s">
-        <v>550</v>
+        <v>557</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
-        <v>551</v>
+        <v>558</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -7225,18 +7322,18 @@
         <v>1</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>552</v>
+        <v>559</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="2" t="s">
-        <v>553</v>
+        <v>560</v>
       </c>
       <c r="B19" s="2">
         <v>3</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>554</v>
+        <v>561</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -7245,96 +7342,96 @@
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2" t="s">
-        <v>555</v>
+        <v>562</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="2" t="s">
-        <v>556</v>
+        <v>563</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2" t="s">
-        <v>557</v>
+        <v>564</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="2" t="s">
-        <v>558</v>
+        <v>565</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2" t="s">
-        <v>559</v>
+        <v>566</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="2" t="s">
-        <v>560</v>
+        <v>567</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="2" t="s">
-        <v>561</v>
+        <v>568</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="2" t="s">
-        <v>562</v>
+        <v>569</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2" t="s">
-        <v>563</v>
+        <v>570</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="2" t="s">
-        <v>564</v>
+        <v>571</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2" t="s">
-        <v>565</v>
+        <v>572</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="2" t="s">
-        <v>566</v>
+        <v>573</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2" t="s">
-        <v>567</v>
+        <v>574</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="2" t="s">
-        <v>568</v>
+        <v>575</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2" t="s">
-        <v>569</v>
+        <v>576</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="2" t="s">
-        <v>570</v>
+        <v>577</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="2" t="s">
-        <v>572</v>
+        <v>579</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="2" t="s">
-        <v>573</v>
+        <v>580</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>572</v>
+        <v>579</v>
       </c>
       <c r="C30" t="s">
-        <v>574</v>
+        <v>581</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clarify stun count stacking and shared duration
</commit_message>
<xml_diff>
--- a/data/excel/Thiết kế game.xlsx
+++ b/data/excel/Thiết kế game.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12180" activeTab="5"/>
+    <workbookView windowWidth="27945" windowHeight="12180" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="Ý tưởng chung" sheetId="1" r:id="rId1"/>
     <sheet name="Giai đoạn phát triên" sheetId="2" r:id="rId2"/>
     <sheet name="Combat mechanic" sheetId="3" r:id="rId3"/>
-    <sheet name="Term" sheetId="4" r:id="rId4"/>
+    <sheet name="Termynology" sheetId="4" r:id="rId4"/>
     <sheet name="dummy Combat power" sheetId="10" r:id="rId5"/>
     <sheet name="Item" sheetId="9" r:id="rId6"/>
     <sheet name="Formula" sheetId="5" r:id="rId7"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="582">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="761" uniqueCount="581">
   <si>
     <t>Tên game</t>
   </si>
@@ -2105,9 +2105,6 @@
   </si>
   <si>
     <t>Allows the character to act, but prevents manual control.</t>
-  </si>
-  <si>
-    <t>Nhân vật vẫn có thể hành động nhưng không thể điều khiển thủ công</t>
   </si>
 </sst>
 </file>
@@ -7153,7 +7150,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="18.7142857142857" customWidth="1"/>
@@ -7319,7 +7316,7 @@
         <v>460</v>
       </c>
       <c r="B18" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>559</v>
@@ -7332,8 +7329,10 @@
       <c r="B19" s="2">
         <v>3</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>561</v>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Has no direct effect. Each target can gain at most 1 Stun Count stack per global turn, regardless of the number of hits or sources. All stacks share a 3-global-turn duration; gaining a stack refreshes the shared duration to 3 global turns. When the duration expires, all stacks reset to 0. Reaching Stun Threshold triggers Stun. Stun Count resets to 0 and cannot increase while stunned.</t>
+        </is>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -7424,14 +7423,6 @@
       <c r="B29" s="2"/>
       <c r="C29" s="2" t="s">
         <v>580</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30" t="s">
-        <v>579</v>
-      </c>
-      <c r="C30" t="s">
-        <v>581</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clarify skills use independent targeting and area rules
</commit_message>
<xml_diff>
--- a/data/excel/Thiết kế game.xlsx
+++ b/data/excel/Thiết kế game.xlsx
@@ -6118,7 +6118,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7142857142857" style="5" customWidth="1"/>
@@ -7075,6 +7075,13 @@
     <row r="48" spans="1:1">
       <c r="A48" s="5" t="s">
         <v>526</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Weapon Attack Target, Area of Attack, and secondary-target Attack modifiers apply only to normal attacks. Each skill defines its own target selection and area of effect and does not inherit these weapon targeting rules or secondary-target Attack modifiers.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update game design workbook
</commit_message>
<xml_diff>
--- a/data/excel/Thiết kế game.xlsx
+++ b/data/excel/Thiết kế game.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12180" activeTab="5"/>
+    <workbookView windowWidth="27945" windowHeight="11460" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Ý tưởng chung" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="894" uniqueCount="626">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="895" uniqueCount="627">
   <si>
     <t>Tên game</t>
   </si>
@@ -1620,7 +1620,7 @@
   </si>
   <si>
     <t>S1.2.2 
-Base MHR +25%</t>
+Deadly strike doesnt require condititon</t>
   </si>
   <si>
     <t>S1.2.3 
@@ -1628,9 +1628,9 @@
   </si>
   <si>
     <t>S1.2.4 
-Base MHR + 15%
+Base MHR + 20%
 Base CHC + 25%
-Base CDB + 70%</t>
+Base CDB + 50%</t>
   </si>
   <si>
     <t>Specialization 2</t>
@@ -1651,15 +1651,15 @@
   </si>
   <si>
     <t>S2.1.2 
-Base SDEF + 350</t>
+Frozen Axe applied Chill, AP recovery -10%, MHR -10%</t>
   </si>
   <si>
     <t>S2.1.3
-Frozen Axe DOT effectiveness +100%</t>
+Frozen Axe DOT effectiveness +200%</t>
   </si>
   <si>
     <t>S2.1.4
-Skill Bluetooth connection effectiveness +20%</t>
+Bluetooth connection effectiveness +20%</t>
   </si>
   <si>
     <t>S2.2.1
@@ -1888,7 +1888,10 @@
     <t>Chill</t>
   </si>
   <si>
-    <t>Reduces AP Recovery and Multi-Hit Rate.</t>
+    <t>Infinity</t>
+  </si>
+  <si>
+    <t>Reduces AP Recovery and Multi-Hit Rate. Stackable. Maximum 5 stacks</t>
   </si>
   <si>
     <t>Break</t>
@@ -2610,7 +2613,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2702,18 +2705,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2727,12 +2718,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -2751,9 +2736,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -3440,7 +3422,7 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="1" ht="61" customHeight="1" spans="1:1">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="58" t="s">
         <v>25</v>
       </c>
     </row>
@@ -4039,79 +4021,79 @@
       </c>
     </row>
     <row r="57" spans="1:3">
-      <c r="A57" s="65" t="s">
+      <c r="A57" s="54" t="s">
         <v>143</v>
       </c>
-      <c r="B57" s="65" t="s">
+      <c r="B57" s="54" t="s">
         <v>144</v>
       </c>
-      <c r="C57" s="65" t="s">
+      <c r="C57" s="54" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="58" customFormat="1" ht="30" customHeight="1" spans="1:3">
-      <c r="A58" s="65" t="s">
+      <c r="A58" s="54" t="s">
         <v>143</v>
       </c>
-      <c r="B58" s="65" t="s">
+      <c r="B58" s="54" t="s">
         <v>146</v>
       </c>
-      <c r="C58" s="65" t="s">
+      <c r="C58" s="54" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="59" customFormat="1" ht="30" customHeight="1" spans="1:3">
-      <c r="A59" s="65" t="s">
+      <c r="A59" s="54" t="s">
         <v>143</v>
       </c>
-      <c r="B59" s="65" t="s">
+      <c r="B59" s="54" t="s">
         <v>148</v>
       </c>
-      <c r="C59" s="65" t="s">
+      <c r="C59" s="54" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="60" customFormat="1" ht="30" customHeight="1" spans="1:3">
-      <c r="A60" s="65" t="s">
+      <c r="A60" s="54" t="s">
         <v>150</v>
       </c>
-      <c r="B60" s="65" t="s">
+      <c r="B60" s="54" t="s">
         <v>151</v>
       </c>
-      <c r="C60" s="65" t="s">
+      <c r="C60" s="54" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="61" customFormat="1" ht="30" customHeight="1" spans="1:3">
-      <c r="A61" s="65" t="s">
+      <c r="A61" s="54" t="s">
         <v>150</v>
       </c>
-      <c r="B61" s="65" t="s">
+      <c r="B61" s="54" t="s">
         <v>153</v>
       </c>
-      <c r="C61" s="65" t="s">
+      <c r="C61" s="54" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="62" customFormat="1" ht="30" customHeight="1" spans="1:3">
-      <c r="A62" s="65" t="s">
+      <c r="A62" s="54" t="s">
         <v>150</v>
       </c>
-      <c r="B62" s="65" t="s">
+      <c r="B62" s="54" t="s">
         <v>155</v>
       </c>
-      <c r="C62" s="65" t="s">
+      <c r="C62" s="54" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="63" customFormat="1" ht="30" customHeight="1" spans="1:3">
-      <c r="A63" s="65" t="s">
+      <c r="A63" s="54" t="s">
         <v>150</v>
       </c>
-      <c r="B63" s="65" t="s">
+      <c r="B63" s="54" t="s">
         <v>157</v>
       </c>
-      <c r="C63" s="65" t="s">
+      <c r="C63" s="54" t="s">
         <v>158</v>
       </c>
     </row>
@@ -5657,12 +5639,12 @@
       </c>
     </row>
     <row r="24" customFormat="1" ht="23.25" customHeight="1" spans="1:1">
-      <c r="A24" s="61" t="s">
+      <c r="A24" s="55" t="s">
         <v>391</v>
       </c>
     </row>
     <row r="26" customFormat="1" ht="18.75" customHeight="1" spans="1:1">
-      <c r="A26" s="62" t="s">
+      <c r="A26" s="56" t="s">
         <v>392</v>
       </c>
     </row>
@@ -5672,57 +5654,57 @@
       </c>
     </row>
     <row r="29" spans="1:1">
-      <c r="A29" s="63" t="s">
+      <c r="A29" s="57" t="s">
         <v>394</v>
       </c>
     </row>
     <row r="30" spans="1:1">
-      <c r="A30" s="63" t="s">
+      <c r="A30" s="57" t="s">
         <v>395</v>
       </c>
     </row>
     <row r="31" spans="1:1">
-      <c r="A31" s="63" t="s">
+      <c r="A31" s="57" t="s">
         <v>396</v>
       </c>
     </row>
     <row r="32" spans="1:1">
-      <c r="A32" s="63" t="s">
+      <c r="A32" s="57" t="s">
         <v>397</v>
       </c>
     </row>
     <row r="33" spans="1:1">
-      <c r="A33" s="63" t="s">
+      <c r="A33" s="57" t="s">
         <v>398</v>
       </c>
     </row>
     <row r="34" spans="1:1">
-      <c r="A34" s="63" t="s">
+      <c r="A34" s="57" t="s">
         <v>399</v>
       </c>
     </row>
     <row r="35" spans="1:1">
-      <c r="A35" s="63" t="s">
+      <c r="A35" s="57" t="s">
         <v>400</v>
       </c>
     </row>
     <row r="36" spans="1:1">
-      <c r="A36" s="63" t="s">
+      <c r="A36" s="57" t="s">
         <v>401</v>
       </c>
     </row>
     <row r="37" spans="1:1">
-      <c r="A37" s="63" t="s">
+      <c r="A37" s="57" t="s">
         <v>402</v>
       </c>
     </row>
     <row r="38" spans="1:1">
-      <c r="A38" s="63" t="s">
+      <c r="A38" s="57" t="s">
         <v>403</v>
       </c>
     </row>
     <row r="40" customFormat="1" ht="18.75" customHeight="1" spans="1:1">
-      <c r="A40" s="62" t="s">
+      <c r="A40" s="56" t="s">
         <v>404</v>
       </c>
     </row>
@@ -5792,7 +5774,7 @@
       </c>
     </row>
     <row r="61" customFormat="1" ht="18.75" customHeight="1" spans="1:1">
-      <c r="A61" s="62" t="s">
+      <c r="A61" s="56" t="s">
         <v>418</v>
       </c>
     </row>
@@ -6029,7 +6011,7 @@
       </c>
     </row>
     <row r="93" customFormat="1" ht="18.75" customHeight="1" spans="1:1">
-      <c r="A93" s="62" t="s">
+      <c r="A93" s="56" t="s">
         <v>459</v>
       </c>
     </row>
@@ -6039,32 +6021,32 @@
       </c>
     </row>
     <row r="97" spans="1:1">
-      <c r="A97" s="63" t="s">
+      <c r="A97" s="57" t="s">
         <v>461</v>
       </c>
     </row>
     <row r="98" spans="1:1">
-      <c r="A98" s="63" t="s">
+      <c r="A98" s="57" t="s">
         <v>462</v>
       </c>
     </row>
     <row r="99" spans="1:1">
-      <c r="A99" s="63" t="s">
+      <c r="A99" s="57" t="s">
         <v>463</v>
       </c>
     </row>
     <row r="100" spans="1:1">
-      <c r="A100" s="63" t="s">
+      <c r="A100" s="57" t="s">
         <v>464</v>
       </c>
     </row>
     <row r="101" spans="1:1">
-      <c r="A101" s="63" t="s">
+      <c r="A101" s="57" t="s">
         <v>465</v>
       </c>
     </row>
     <row r="102" spans="1:1">
-      <c r="A102" s="63" t="s">
+      <c r="A102" s="57" t="s">
         <v>466</v>
       </c>
     </row>
@@ -6089,7 +6071,7 @@
       </c>
     </row>
     <row r="110" customFormat="1" ht="18.75" customHeight="1" spans="1:1">
-      <c r="A110" s="62" t="s">
+      <c r="A110" s="56" t="s">
         <v>469</v>
       </c>
     </row>
@@ -6403,7 +6385,7 @@
         <v>207</v>
       </c>
       <c r="B14" s="34">
-        <f>SUM(C14,E14)</f>
+        <f t="shared" si="0"/>
         <v>1.2</v>
       </c>
       <c r="C14" s="34">
@@ -6527,7 +6509,7 @@
         <v>191</v>
       </c>
       <c r="B18" s="31">
-        <f>SUM(C18,E18)</f>
+        <f t="shared" si="0"/>
         <v>70</v>
       </c>
       <c r="C18" s="31">
@@ -6802,7 +6784,7 @@
       <c r="J28" s="38" t="s">
         <v>493</v>
       </c>
-      <c r="K28" s="56" t="s">
+      <c r="K28" s="39" t="s">
         <v>494</v>
       </c>
     </row>
@@ -6838,7 +6820,7 @@
       <c r="J29" s="38" t="s">
         <v>500</v>
       </c>
-      <c r="K29" s="56">
+      <c r="K29" s="39">
         <f>4.8*1000*2%*5</f>
         <v>480</v>
       </c>
@@ -6858,7 +6840,7 @@
       <c r="J30" s="38" t="s">
         <v>500</v>
       </c>
-      <c r="K30" s="56">
+      <c r="K30" s="39">
         <f>4.8*1000*2%*5</f>
         <v>480</v>
       </c>
@@ -6893,188 +6875,188 @@
       <c r="J31" s="44" t="s">
         <v>506</v>
       </c>
-      <c r="K31" s="57">
+      <c r="K31" s="40">
         <f>4.8*1000*70%*5</f>
         <v>16800</v>
       </c>
     </row>
     <row r="32" ht="30" spans="1:11">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="38" t="s">
         <v>507</v>
       </c>
-      <c r="B32" s="47" t="s">
+      <c r="B32" s="38" t="s">
         <v>508</v>
       </c>
-      <c r="C32" s="48">
+      <c r="C32" s="41">
         <v>800</v>
       </c>
-      <c r="D32" s="49">
+      <c r="D32" s="42">
         <v>0</v>
       </c>
-      <c r="E32" s="47" t="s">
+      <c r="E32" s="38" t="s">
         <v>509</v>
       </c>
-      <c r="F32" s="47" t="s">
+      <c r="F32" s="38" t="s">
         <v>510</v>
       </c>
-      <c r="G32" s="47" t="s">
+      <c r="G32" s="38" t="s">
         <v>504</v>
       </c>
-      <c r="H32" s="49">
+      <c r="H32" s="42">
         <v>2</v>
       </c>
-      <c r="I32" s="47" t="s">
+      <c r="I32" s="38" t="s">
         <v>511</v>
       </c>
-      <c r="J32" s="47" t="s">
+      <c r="J32" s="38" t="s">
         <v>512</v>
       </c>
-      <c r="K32" s="58">
+      <c r="K32" s="52">
         <f>10%*5</f>
         <v>0.5</v>
       </c>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="47"/>
-      <c r="B33" s="47"/>
-      <c r="C33" s="48"/>
-      <c r="D33" s="49"/>
-      <c r="E33" s="47"/>
-      <c r="F33" s="47"/>
-      <c r="G33" s="47"/>
-      <c r="H33" s="49"/>
-      <c r="I33" s="47" t="s">
+      <c r="A33" s="38"/>
+      <c r="B33" s="38"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="42"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="38"/>
+      <c r="H33" s="42"/>
+      <c r="I33" s="38" t="s">
         <v>513</v>
       </c>
-      <c r="J33" s="47" t="s">
+      <c r="J33" s="38" t="s">
         <v>514</v>
       </c>
-      <c r="K33" s="59">
+      <c r="K33" s="53">
         <f>6%*5</f>
         <v>0.3</v>
       </c>
     </row>
     <row r="34" ht="43" customHeight="1" spans="1:11">
-      <c r="A34" s="47"/>
-      <c r="B34" s="47"/>
-      <c r="C34" s="48"/>
-      <c r="D34" s="49"/>
-      <c r="E34" s="47"/>
-      <c r="F34" s="47"/>
-      <c r="G34" s="47"/>
-      <c r="H34" s="49"/>
-      <c r="I34" s="47" t="s">
+      <c r="A34" s="38"/>
+      <c r="B34" s="38"/>
+      <c r="C34" s="41"/>
+      <c r="D34" s="42"/>
+      <c r="E34" s="38"/>
+      <c r="F34" s="38"/>
+      <c r="G34" s="38"/>
+      <c r="H34" s="42"/>
+      <c r="I34" s="38" t="s">
         <v>515</v>
       </c>
-      <c r="J34" s="47" t="s">
+      <c r="J34" s="38" t="s">
         <v>516</v>
       </c>
-      <c r="K34" s="59">
+      <c r="K34" s="53">
         <f>3%*5</f>
         <v>0.15</v>
       </c>
     </row>
     <row r="36" ht="45" spans="1:8">
-      <c r="A36" s="50" t="s">
+      <c r="A36" s="47" t="s">
         <v>517</v>
       </c>
-      <c r="B36" s="50" t="s">
+      <c r="B36" s="47" t="s">
         <v>518</v>
       </c>
-      <c r="C36" s="50" t="s">
+      <c r="C36" s="47" t="s">
         <v>519</v>
       </c>
-      <c r="D36" s="50" t="s">
+      <c r="D36" s="47" t="s">
         <v>520</v>
       </c>
-      <c r="E36" s="51" t="s">
+      <c r="E36" s="47" t="s">
         <v>521</v>
       </c>
-      <c r="F36" s="51" t="s">
+      <c r="F36" s="47" t="s">
         <v>522</v>
       </c>
-      <c r="G36" s="51" t="s">
+      <c r="G36" s="47" t="s">
         <v>523</v>
       </c>
-      <c r="H36" s="51" t="s">
+      <c r="H36" s="47" t="s">
         <v>524</v>
       </c>
     </row>
     <row r="37" ht="60" spans="1:8">
-      <c r="A37" s="50"/>
-      <c r="B37" s="50"/>
-      <c r="C37" s="50"/>
-      <c r="D37" s="50"/>
-      <c r="E37" s="51" t="s">
+      <c r="A37" s="47"/>
+      <c r="B37" s="47"/>
+      <c r="C37" s="47"/>
+      <c r="D37" s="47"/>
+      <c r="E37" s="47" t="s">
         <v>525</v>
       </c>
-      <c r="F37" s="51" t="s">
+      <c r="F37" s="47" t="s">
         <v>526</v>
       </c>
-      <c r="G37" s="51" t="s">
+      <c r="G37" s="47" t="s">
         <v>527</v>
       </c>
-      <c r="H37" s="51" t="s">
+      <c r="H37" s="47" t="s">
         <v>528</v>
       </c>
     </row>
     <row r="38" spans="1:8">
-      <c r="A38" s="52"/>
-      <c r="B38" s="52"/>
-      <c r="C38" s="52"/>
-      <c r="D38" s="52"/>
-      <c r="E38" s="53"/>
-      <c r="F38" s="53"/>
-      <c r="G38" s="53"/>
-      <c r="H38" s="53"/>
+      <c r="A38" s="48"/>
+      <c r="B38" s="48"/>
+      <c r="C38" s="48"/>
+      <c r="D38" s="48"/>
+      <c r="E38" s="49"/>
+      <c r="F38" s="49"/>
+      <c r="G38" s="49"/>
+      <c r="H38" s="49"/>
     </row>
     <row r="39" ht="60" spans="1:10">
-      <c r="A39" s="54" t="s">
+      <c r="A39" s="50" t="s">
         <v>529</v>
       </c>
-      <c r="B39" s="54" t="s">
+      <c r="B39" s="50" t="s">
         <v>530</v>
       </c>
-      <c r="C39" s="54" t="s">
+      <c r="C39" s="50" t="s">
         <v>531</v>
       </c>
-      <c r="D39" s="54" t="s">
+      <c r="D39" s="50" t="s">
         <v>532</v>
       </c>
-      <c r="E39" s="51" t="s">
+      <c r="E39" s="47" t="s">
         <v>533</v>
       </c>
-      <c r="F39" s="51" t="s">
+      <c r="F39" s="47" t="s">
         <v>534</v>
       </c>
-      <c r="G39" s="51" t="s">
+      <c r="G39" s="47" t="s">
         <v>535</v>
       </c>
-      <c r="H39" s="51" t="s">
+      <c r="H39" s="47" t="s">
         <v>536</v>
       </c>
-      <c r="I39" s="60"/>
-      <c r="J39" s="60"/>
+      <c r="I39" s="54"/>
+      <c r="J39" s="54"/>
     </row>
     <row r="40" ht="60" spans="1:10">
-      <c r="A40" s="55"/>
-      <c r="B40" s="55"/>
-      <c r="C40" s="55"/>
-      <c r="D40" s="55"/>
-      <c r="E40" s="51" t="s">
+      <c r="A40" s="51"/>
+      <c r="B40" s="51"/>
+      <c r="C40" s="51"/>
+      <c r="D40" s="51"/>
+      <c r="E40" s="47" t="s">
         <v>537</v>
       </c>
-      <c r="F40" s="51" t="s">
+      <c r="F40" s="47" t="s">
         <v>538</v>
       </c>
-      <c r="G40" s="50" t="s">
+      <c r="G40" s="47" t="s">
         <v>539</v>
       </c>
-      <c r="H40" s="51" t="s">
+      <c r="H40" s="47" t="s">
         <v>540</v>
       </c>
-      <c r="I40" s="60"/>
-      <c r="J40" s="60"/>
+      <c r="I40" s="54"/>
+      <c r="J40" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="24">
@@ -8467,64 +8449,67 @@
       <c r="A22" t="s">
         <v>610</v>
       </c>
+      <c r="B22" t="s">
+        <v>611</v>
+      </c>
       <c r="C22" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="C23" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="C24" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="C25" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="C26" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="C27" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="C28" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="C29" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add reusable combat simulation runner and configuration
</commit_message>
<xml_diff>
--- a/data/excel/Thiết kế game.xlsx
+++ b/data/excel/Thiết kế game.xlsx
@@ -1966,12 +1966,13 @@
   </si>
   <si>
     <t>S1.1.1
-Atk + 20%</t>
+Atk + 10%
+Base MHR +10%</t>
   </si>
   <si>
     <t>S1.1.2 
 Base Acc +20%
-Multi-hit rate +10%</t>
+Base MHR +10%</t>
   </si>
   <si>
     <t>S1.1.3
@@ -7979,7 +7980,7 @@
       </c>
       <c r="B11" s="30">
         <f t="shared" si="0"/>
-        <v>2909.52380952381</v>
+        <v>2909.5238095238</v>
       </c>
       <c r="C11" s="30">
         <f>6840/G11</f>
@@ -8522,11 +8523,11 @@
         <v>618</v>
       </c>
       <c r="B30" s="37">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="C30" s="37">
-        <f>2*1000*2</f>
-        <v>4000</v>
+        <f>2*1000*2*1.3</f>
+        <v>5200</v>
       </c>
       <c r="D30" s="37">
         <v>10</v>
@@ -8565,7 +8566,7 @@
         <v>800</v>
       </c>
       <c r="D31" s="39">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E31" s="39" t="s">
         <v>624</v>

</xml_diff>

<commit_message>
Clarify damage penalties and cooldown timing; recalculate Soldier mana
</commit_message>
<xml_diff>
--- a/data/excel/Thiết kế game.xlsx
+++ b/data/excel/Thiết kế game.xlsx
@@ -7166,7 +7166,8 @@
         <v>125</v>
       </c>
       <c r="C32" s="36">
-        <v>7583</v>
+        <f>ROUND(4106*(50.5*4147.2+66.5*8270+66*L32)/1239658.6,0)</f>
+        <v>9385</v>
       </c>
       <c r="D32" s="14">
         <v>4</v>
@@ -7247,7 +7248,8 @@
         <v>100</v>
       </c>
       <c r="C35" s="36">
-        <v>5748</v>
+        <f>ROUND(4106*(67*4147.2+67*8270+66*L35)/1239658.6,0)</f>
+        <v>7219</v>
       </c>
       <c r="D35" s="14">
         <v>5</v>
@@ -7265,16 +7267,18 @@
       <c r="I35" s="13" t="s">
         <v>464</v>
       </c>
-      <c r="J35" s="13" t="s">
-        <v>1147</v>
+      <c r="J35" s="13" t="inlineStr">
+        <is>
+          <t>1.654*1000*SL</t>
+        </is>
       </c>
       <c r="K35" s="64">
         <f>1.654*1000*5</f>
         <v>8270</v>
       </c>
       <c r="L35" s="65">
-        <f>8279*1.975*1.25</f>
-        <v>20438.78125</v>
+        <f>8270*1.975*1.25</f>
+        <v>20416.5625</v>
       </c>
     </row>
     <row r="36" s="52" customFormat="1" ht="32" customHeight="1" spans="1:12">
@@ -10911,8 +10915,10 @@
       <c r="B9" s="147" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="147" t="s">
-        <v>39</v>
+      <c r="C9" s="147" t="inlineStr">
+        <is>
+          <t>Initialize each skill's remaining cooldown to its applicable cooldown duration, unless an explicit effect overrides it. Both teams begin cooldown recovery at the end of global turn 1, even if their first team turn has not occurred.</t>
+        </is>
       </c>
     </row>
     <row r="10" ht="30" spans="1:3">
@@ -11917,8 +11923,10 @@
       <c r="B103" s="147" t="s">
         <v>229</v>
       </c>
-      <c r="C103" s="147" t="s">
-        <v>230</v>
+      <c r="C103" s="147" t="inlineStr">
+        <is>
+          <t>For a landed hit, use zero mitigation if Penetration succeeds; otherwise use the target's Final Defense mitigation. A critical hit multiplies damage by 1 + Final Critical Damage Bonus. Resolve applicable damage adjustments for each recipient, then multiply secondary-target final damage by (1 - Sub-target Damage Penalty). This penalty does not reduce Attack.</t>
+        </is>
       </c>
     </row>
     <row r="104" ht="30" spans="1:3">
@@ -12122,8 +12130,10 @@
       <c r="B122" s="147" t="s">
         <v>272</v>
       </c>
-      <c r="C122" s="147" t="s">
-        <v>273</v>
+      <c r="C122" s="147" t="inlineStr">
+        <is>
+          <t>At the end of every global turn, starting with global turn 1, apply default cooldown recovery to both teams. The team acting second also receives recovery at the end of global turn 1; a skill initialized with cooldown 1 is therefore ready on global turn 2, subject to its other casting requirements.</t>
+        </is>
       </c>
     </row>
     <row r="123" spans="1:3">
@@ -14158,7 +14168,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:R176"/>
+  <dimension ref="A1:R186"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7142857142857" customWidth="1"/>
@@ -15875,8 +15885,73 @@
       </c>
     </row>
     <row r="176" spans="1:1">
-      <c r="A176" t="s">
-        <v>839</v>
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Mana reference: active SATK 8,270 without Stun Count; AP cost 100; mana cost 4,106; cooldown 3 global turns. CP/stat and status pricing retain the separate 5,800-SATK +1-Stun-Count reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Mana timing: evaluate 200 own team turns for each starting order. Both teams recover cooldown at the end of global turn 1. Start with 0 AP; recover 100 AP per own team turn; ignore MP exhaustion for pricing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Action priority: skill being priced, then reference active, then normal attack. Do not recast while the skill duration remains active. Apply listed AP costs and ordinary action-slot eligibility; a completed expensive action may leave AP negative.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Reference totals: acting first gives 101 normals + 99 actives = 1,237,597.20 SATK equivalent; acting second gives 100 normals + 100 actives = 1,241,720.00. Mean reference value = 1,239,658.60.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Mana Cost = 4,106 * Mean Total SATK Equivalent With Skill / 1,239,658.60. Average both starting orders. Skill SATK equivalent already includes assigned effects and area value; do not apply them again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>War Cry: AP 125, cooldown 4, duration 6, SATK equivalent 31,426. First: 51 normals, 66 reference actives, 66 War Cry casts, 17 skipped turns. Second: 50 normals, 67 reference actives, 66 War Cry casts, 17 skipped turns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>War Cry: mean total value 2,833,504.60; mana 9,385.140302; selected cost 9,385 MP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>God-King Slayer: AP 100, cooldown 5, instant; SATK equivalent = 8,270 * 1.975 * 1.25 = 20,416.5625. Both starting orders give 67 normals, 67 reference actives and 66 God-King Slayer casts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>God-King Slayer: total value 2,179,445.525; mana 7,218.764364; selected cost 7,219 MP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>These two Soldier mana costs use the updated cooldown timing and both starting orders. Other character mana entries have not been recalculated in this revision. Action counts are fixed for the listed AP costs, cooldowns and durations; recalculate them when those inputs change.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -16953,8 +17028,10 @@
       </c>
     </row>
     <row r="51" spans="1:1">
-      <c r="A51" s="91" t="s">
-        <v>873</v>
+      <c r="A51" s="91" t="inlineStr">
+        <is>
+          <t>Calculate damage separately against each recipient using its own mitigation and applicable damage modifiers. Then apply the listed Sub-target Damage Penalty to the secondary target's final damage: Final Sub-target Damage = Final Damage Before This Penalty * (1 - Penalty). A 50% penalty leaves 50% damage; a 75% penalty leaves 25%. This penalty does not reduce Attack or SATK. The primary target receives no sub-target penalty.</t>
+        </is>
       </c>
     </row>
     <row r="52" spans="1:1">
@@ -16973,8 +17050,10 @@
       </c>
     </row>
     <row r="55" spans="1:1">
-      <c r="A55" t="s">
-        <v>877</v>
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Weapon Attack Target, Area of Attack, and Sub-target Damage Penalty apply only to normal attacks. Each skill defines its own targeting, area, and sub-target damage penalty; weapon rules are not inherited unless the skill explicitly states otherwise.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Document CP review under global-turn-one cooldown recovery
</commit_message>
<xml_diff>
--- a/data/excel/Thiết kế game.xlsx
+++ b/data/excel/Thiết kế game.xlsx
@@ -5473,7 +5473,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="150">
+  <cellXfs count="154">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -5838,6 +5838,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment wrapText="1" vertical="top"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment wrapText="1" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -14168,7 +14177,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:R186"/>
+  <dimension ref="A1:R206"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7142857142857" customWidth="1"/>
@@ -15954,7 +15963,239 @@
         </is>
       </c>
     </row>
+    <row r="188" ht="28" customHeight="1">
+      <c r="A188" s="151" t="inlineStr">
+        <is>
+          <t>8. CP Review — Cooldown Recovery from Global Turn 1 — 2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="44" customHeight="1">
+      <c r="A189" s="151" t="inlineStr">
+        <is>
+          <t>Decision: keep all selected CP per stat and status coefficients. Analytic magnitude prices and explicit budget conventions are unchanged. The two new stun estimates differ from selected prices by less than 2%; retain 1,850 and 9,600 CP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="42" customHeight="1">
+      <c r="A190" s="151" t="inlineStr">
+        <is>
+          <t>Stat / tested increase</t>
+        </is>
+      </c>
+      <c r="B190" s="151" t="inlineStr">
+        <is>
+          <t>Selected CP</t>
+        </is>
+      </c>
+      <c r="C190" s="151" t="inlineStr">
+        <is>
+          <t>Old timing test</t>
+        </is>
+      </c>
+      <c r="D190" s="151" t="inlineStr">
+        <is>
+          <t>New timing test</t>
+        </is>
+      </c>
+      <c r="E190" s="151" t="inlineStr">
+        <is>
+          <t>New minus selected</t>
+        </is>
+      </c>
+      <c r="F190" s="151" t="inlineStr">
+        <is>
+          <t>Change vs selected</t>
+        </is>
+      </c>
+      <c r="G190" s="151" t="inlineStr">
+        <is>
+          <t>New estimate 95% interval</t>
+        </is>
+      </c>
+      <c r="H190" s="151" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="44" customHeight="1">
+      <c r="A191" s="151" t="inlineStr">
+        <is>
+          <t>Stun Threshold: 4 to 5</t>
+        </is>
+      </c>
+      <c r="B191" s="152">
+        <v>1850</v>
+      </c>
+      <c r="C191" s="152">
+        <v>1969.0</v>
+      </c>
+      <c r="D191" s="152">
+        <v>1866.0</v>
+      </c>
+      <c r="E191" s="152">
+        <f>D191-B191</f>
+        <v>16.0</v>
+      </c>
+      <c r="F191" s="153">
+        <f>E191/B191</f>
+        <v>0.008648648648648649</v>
+      </c>
+      <c r="G191" s="151" t="inlineStr">
+        <is>
+          <t>1,577.34 to 2,154.66</t>
+        </is>
+      </c>
+      <c r="H191" s="151" t="inlineStr">
+        <is>
+          <t>Keep selected CP</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="44" customHeight="1">
+      <c r="A192" s="151" t="inlineStr">
+        <is>
+          <t>Attack Stun Count: 0 to 1</t>
+        </is>
+      </c>
+      <c r="B192" s="152">
+        <v>9600</v>
+      </c>
+      <c r="C192" s="152">
+        <v>9702.0</v>
+      </c>
+      <c r="D192" s="152">
+        <v>9444.0</v>
+      </c>
+      <c r="E192" s="152">
+        <f>D192-B192</f>
+        <v>-156.0</v>
+      </c>
+      <c r="F192" s="153">
+        <f>E192/B192</f>
+        <v>-0.01625</v>
+      </c>
+      <c r="G192" s="151" t="inlineStr">
+        <is>
+          <t>9,115.55 to 9,772.45</t>
+        </is>
+      </c>
+      <c r="H192" s="151" t="inlineStr">
+        <is>
+          <t>Keep selected CP</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="44" customHeight="1">
+      <c r="A194" s="151" t="inlineStr">
+        <is>
+          <t>Comparison design: 100 battles per configuration, 50 per starting order, matched seed base 20261026. Use per-side/action random streams. CP = mean paired change in (A remaining HP - B remaining HP), with 1 HP = 1 CP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="44" customHeight="1">
+      <c r="A195" s="151" t="inlineStr">
+        <is>
+          <t>Current-timing sensitivity tests: HP 50,000; MP 41,060; active SATK 5,800, AP 100, MP cost 4,106, cooldown 3; passive Attack Effectiveness +20%. Normal-first alternating completed actions; normal fallback if active unavailable. Same rules except initial cooldown recovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" ht="44" customHeight="1">
+      <c r="A196" s="151" t="inlineStr">
+        <is>
+          <t>Threshold test: only B applies stun, through normal and active count 1; A threshold changes 4 to 5. Normal-count test: only A applies stun; A active count stays 1 and normal count changes 0 to 1. Stun/count duration 3 global turns; one stack per target per global turn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="197" ht="44" customHeight="1">
+      <c r="A197" s="151" t="inlineStr">
+        <is>
+          <t>Original benchmark reproduction (no cooldown/MP limits): threshold 1,852.00 CP and normal count 9,579.00 CP, exactly reproducing the original results. The original selected prices remain 1,850 and 9,600. Do not confuse this unrestricted benchmark with the additional cooldown-constrained tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198" ht="44" customHeight="1">
+      <c r="A198" s="151" t="inlineStr">
+        <is>
+          <t>Cooldown-rule-only effect with CD/MP fixed: threshold 1,969 -&gt; 1,866 CP (-103.00; approx. 95% paired interval -265.69 to +59.69). Normal count 9,702 -&gt; 9,444 CP (-258.00; interval -501.94 to -14.06). The latter indicates a small timing effect in this sample; it does not justify replacing the selected 9,600 budget with a precise sample estimate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199" ht="44" customHeight="1">
+      <c r="A199" s="151" t="inlineStr">
+        <is>
+          <t>Uncertainty: approximate 95% intervals use 1.984 times the standard error from 100 paired trials. Both current selected prices lie within the intervals of the corresponding new estimates. Samples are reference-scenario evidence, not universal prices for all characters or teams.</t>
+        </is>
+      </c>
+    </row>
+    <row r="200" ht="44" customHeight="1">
+      <c r="A200" s="151" t="inlineStr">
+        <is>
+          <t>Analytic stat prices unchanged: HP, MP package, Attack, Defense, Skill Defense, MHR, Penetration, CHC, CDB, Skill Points package, Evasion, Healing Amplification, Block Chance and Counterattack Chance. AP Recovery and Accuracy retain their explicit budget conventions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201" ht="44" customHeight="1">
+      <c r="A201" s="151" t="inlineStr">
+        <is>
+          <t>Status coefficients unchanged: Rage/Intimidated, Calm/Weaken, Fortify/Sunder, Resistance/Exposure, Haste/Slow, Onslaught/Falter, Blind, Precision/Doubt, Shield, Block Chance, Counterattack Chance, Vulnerable/Durable, Chill and Break. These price magnitude, not duration or actual cast counts. Blank coefficients remain unpriced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="202" ht="44" customHeight="1">
+      <c r="A202" s="151" t="inlineStr">
+        <is>
+          <t>Why formulas do not change: the CP reference remains one normal action alternating with one active, with mixed damage 2,486.80 per completed action. It excludes initial cooldown delays. Changing this reference to a finite combat schedule would be a separate repricing decision, not an automatic consequence of the new cooldown rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203" ht="44" customHeight="1">
+      <c r="A203" s="151" t="inlineStr">
+        <is>
+          <t>Cadence check without stun or MP exhaustion, active-first when ready: over 20 own turns, old timing gives 11 normals + 9 actives for either starting side. New timing gives 11 + 9 for the first side, 10 + 10 for the second. Average damage changes 2,445.48 -&gt; 2,466.14 (+0.84%). This diagnostic is not the selected 2,486.80 magnitude reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204" ht="44" customHeight="1">
+      <c r="A204" s="151" t="inlineStr">
+        <is>
+          <t>Over 200 own turns, the analogous damage diagnostic changes 2,482.668 -&gt; 2,484.734 (+0.08%). This check excludes MP exhaustion; MP pricing itself retains the separate 10-usable-cast package assumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" ht="44" customHeight="1">
+      <c r="A205" s="151" t="inlineStr">
+        <is>
+          <t>Engine validation: confirmed that both teams recover cooldown at end of global turn 1; a cooldown-1 skill is ready for the second team on global turn 2. Duration/count expiration and cooldown assigned on casting remain unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="206" ht="44" customHeight="1">
+      <c r="A206" s="151" t="inlineStr">
+        <is>
+          <t>Source audit: the original simulation-based coefficients excluded mana/cooldown. New tests supplement, rather than silently replace, those valuation assumptions. No character stats, skill mana costs, spec nodes or selected CP totals are changed in this review.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="A188:H188"/>
+    <mergeCell ref="A189:H189"/>
+    <mergeCell ref="A194:H194"/>
+    <mergeCell ref="A195:H195"/>
+    <mergeCell ref="A196:H196"/>
+    <mergeCell ref="A197:H197"/>
+    <mergeCell ref="A198:H198"/>
+    <mergeCell ref="A199:H199"/>
+    <mergeCell ref="A200:H200"/>
+    <mergeCell ref="A201:H201"/>
+    <mergeCell ref="A202:H202"/>
+    <mergeCell ref="A203:H203"/>
+    <mergeCell ref="A204:H204"/>
+    <mergeCell ref="A205:H205"/>
+    <mergeCell ref="A206:H206"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>
@@ -17815,16 +18056,20 @@
       <c r="A57" s="86" t="s">
         <v>991</v>
       </c>
-      <c r="B57" s="86" t="s">
-        <v>992</v>
+      <c r="B57" s="86" t="inlineStr">
+        <is>
+          <t>These coefficients price effect magnitude. They exclude duration, uptime, recipient count, cast frequency, and resource costs. They are independent of the 200-team-turn mana-cost method. Stun value is not added to the mixed-damage denominator. Reviewed 2026-10-29 after the global-turn-1 cooldown change: coefficients retained; see Balanced Dummy section 8.</t>
+        </is>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="86" t="s">
         <v>993</v>
       </c>
-      <c r="B58" s="86" t="s">
-        <v>994</v>
+      <c r="B58" s="86" t="inlineStr">
+        <is>
+          <t>Each +1 active SATK adds 0.25 mixed damage. CP per SATK = 50,000 * 0.25 / 2,486.80 = 5.02654013. Point per 100 CP = 19.8944. Modifier per 100 CP = 19.8944 / 5,800 = 0.34300690%. This prices the SATK increase only; the skill keeps +1 Stun Count. SATK is not an additional basic-stat CP entry.</t>
+        </is>
       </c>
     </row>
     <row r="59" spans="1:2">

</xml_diff>